<commit_message>
Add comprehensive BA onboarding documentation
Add detailed business analyst onboarding documentation covering system architecture, modules, workflows, and business logic.

Includes:
- Backend module deep-dives (CRM, TradeSpend, ProductSpecs, DataHub, Broker, etc.)
- Frontend application maps and role-based routing
- Entity relationships, glossary, and permission matrix
- End-to-end workflow walkthroughs
- Known gaps, risks, and inconsistencies
- Deliverable/issue documentation (CS-1318, CS-1324, CS-1417, CS-1423, CS-1431, CS-1433, CS-1436)

Documentation is code-grounded with file/line citations for verification. Includes both backend and frontend repositories.
</commit_message>
<xml_diff>
--- a/Caboodle_Backlog_by_Module.xlsx
+++ b/Caboodle_Backlog_by_Module.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/db8adb1db0cd9913/Desktop/CaboodleServices/A IT/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\My Code\Caboodle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="164" documentId="8_{57C4FD4B-B8F1-456C-968C-326B1C173EE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA8EE6D2-E9F9-4B94-93D6-2999F2FD31BF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{300B3427-E2C9-4FDF-ACD9-0759C256B6C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -2846,7 +2846,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -3017,15 +3017,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="22" fontId="0" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3050,6 +3041,19 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3328,197 +3332,197 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
     </row>
     <row r="3" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
     </row>
     <row r="4" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="67" t="s">
+      <c r="B4" s="77" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="67"/>
-      <c r="D4" s="67"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="67"/>
+      <c r="C4" s="77"/>
+      <c r="D4" s="77"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="67"/>
-      <c r="C5" s="67"/>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="77"/>
+      <c r="D5" s="77"/>
+      <c r="E5" s="77"/>
+      <c r="F5" s="77"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="67"/>
-      <c r="C6" s="67"/>
-      <c r="D6" s="67"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="67"/>
+      <c r="B6" s="77"/>
+      <c r="C6" s="77"/>
+      <c r="D6" s="77"/>
+      <c r="E6" s="77"/>
+      <c r="F6" s="77"/>
     </row>
     <row r="7" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="67" t="s">
+      <c r="B7" s="77" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="67"/>
-      <c r="D7" s="67"/>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
+      <c r="C7" s="77"/>
+      <c r="D7" s="77"/>
+      <c r="E7" s="77"/>
+      <c r="F7" s="77"/>
     </row>
     <row r="8" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="67" t="s">
+      <c r="B8" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="67"/>
-      <c r="D8" s="67"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="67"/>
+      <c r="C8" s="77"/>
+      <c r="D8" s="77"/>
+      <c r="E8" s="77"/>
+      <c r="F8" s="77"/>
     </row>
     <row r="9" spans="1:6" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="67" t="s">
+      <c r="B9" s="77" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="67"/>
-      <c r="D9" s="67"/>
-      <c r="E9" s="67"/>
-      <c r="F9" s="67"/>
+      <c r="C9" s="77"/>
+      <c r="D9" s="77"/>
+      <c r="E9" s="77"/>
+      <c r="F9" s="77"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="67"/>
-      <c r="C10" s="67"/>
-      <c r="D10" s="67"/>
-      <c r="E10" s="67"/>
-      <c r="F10" s="67"/>
+      <c r="B10" s="77"/>
+      <c r="C10" s="77"/>
+      <c r="D10" s="77"/>
+      <c r="E10" s="77"/>
+      <c r="F10" s="77"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="67"/>
-      <c r="C11" s="67"/>
-      <c r="D11" s="67"/>
-      <c r="E11" s="67"/>
-      <c r="F11" s="67"/>
+      <c r="B11" s="77"/>
+      <c r="C11" s="77"/>
+      <c r="D11" s="77"/>
+      <c r="E11" s="77"/>
+      <c r="F11" s="77"/>
     </row>
     <row r="12" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="67" t="s">
+      <c r="B12" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="67"/>
-      <c r="D12" s="67"/>
-      <c r="E12" s="67"/>
-      <c r="F12" s="67"/>
+      <c r="C12" s="77"/>
+      <c r="D12" s="77"/>
+      <c r="E12" s="77"/>
+      <c r="F12" s="77"/>
     </row>
     <row r="13" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="67" t="s">
+      <c r="B13" s="77" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="67"/>
-      <c r="D13" s="67"/>
-      <c r="E13" s="67"/>
-      <c r="F13" s="67"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="77"/>
+      <c r="F13" s="77"/>
     </row>
     <row r="14" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="67" t="s">
+      <c r="B14" s="77" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="67"/>
-      <c r="D14" s="67"/>
-      <c r="E14" s="67"/>
-      <c r="F14" s="67"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="77"/>
+      <c r="E14" s="77"/>
+      <c r="F14" s="77"/>
     </row>
     <row r="15" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="67" t="s">
+      <c r="B15" s="77" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="67"/>
-      <c r="D15" s="67"/>
-      <c r="E15" s="67"/>
-      <c r="F15" s="67"/>
+      <c r="C15" s="77"/>
+      <c r="D15" s="77"/>
+      <c r="E15" s="77"/>
+      <c r="F15" s="77"/>
     </row>
     <row r="16" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="67" t="s">
+      <c r="B16" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="67"/>
-      <c r="D16" s="67"/>
-      <c r="E16" s="67"/>
-      <c r="F16" s="67"/>
+      <c r="C16" s="77"/>
+      <c r="D16" s="77"/>
+      <c r="E16" s="77"/>
+      <c r="F16" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B10:F10"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -3546,21 +3550,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="78" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -5263,7 +5267,7 @@
       <c r="B1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C1" s="70" t="s">
+      <c r="C1" s="67" t="s">
         <v>72</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -13999,7 +14003,7 @@
       <c r="B227" s="50" t="s">
         <v>205</v>
       </c>
-      <c r="C227" s="71" t="s">
+      <c r="C227" s="68" t="s">
         <v>798</v>
       </c>
       <c r="D227" s="51" t="s">
@@ -14035,7 +14039,7 @@
       <c r="B228" s="50" t="s">
         <v>205</v>
       </c>
-      <c r="C228" s="71" t="s">
+      <c r="C228" s="68" t="s">
         <v>799</v>
       </c>
       <c r="D228" s="51" t="s">
@@ -14071,7 +14075,7 @@
       <c r="B229" s="50" t="s">
         <v>266</v>
       </c>
-      <c r="C229" s="71" t="s">
+      <c r="C229" s="68" t="s">
         <v>800</v>
       </c>
       <c r="D229" s="51" t="s">
@@ -14107,7 +14111,7 @@
       <c r="B230" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="C230" s="71" t="s">
+      <c r="C230" s="68" t="s">
         <v>801</v>
       </c>
       <c r="D230" s="51" t="s">
@@ -14143,7 +14147,7 @@
       <c r="B231" s="50" t="s">
         <v>100</v>
       </c>
-      <c r="C231" s="71" t="s">
+      <c r="C231" s="68" t="s">
         <v>802</v>
       </c>
       <c r="D231" s="51" t="s">
@@ -14179,7 +14183,7 @@
       <c r="B232" s="50" t="s">
         <v>100</v>
       </c>
-      <c r="C232" s="71" t="s">
+      <c r="C232" s="68" t="s">
         <v>824</v>
       </c>
       <c r="D232" s="52" t="s">
@@ -14201,10 +14205,10 @@
       <c r="J232" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="K232" s="69">
+      <c r="K232" s="66">
         <v>46211.036805555559</v>
       </c>
-      <c r="L232" s="69">
+      <c r="L232" s="66">
         <v>46211.036805555559</v>
       </c>
     </row>
@@ -14215,7 +14219,7 @@
       <c r="B233" s="50" t="s">
         <v>100</v>
       </c>
-      <c r="C233" s="71" t="s">
+      <c r="C233" s="68" t="s">
         <v>826</v>
       </c>
       <c r="D233" s="52" t="s">
@@ -14237,10 +14241,10 @@
       <c r="J233" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="K233" s="69">
+      <c r="K233" s="66">
         <v>46210.98541666667</v>
       </c>
-      <c r="L233" s="69">
+      <c r="L233" s="66">
         <v>46210.98541666667</v>
       </c>
     </row>
@@ -14251,7 +14255,7 @@
       <c r="B234" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="C234" s="71" t="s">
+      <c r="C234" s="68" t="s">
         <v>828</v>
       </c>
       <c r="D234" s="52" t="s">
@@ -14273,10 +14277,10 @@
       <c r="J234" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="K234" s="69">
+      <c r="K234" s="66">
         <v>46210.981944444444</v>
       </c>
-      <c r="L234" s="69">
+      <c r="L234" s="66">
         <v>46210.981944444444</v>
       </c>
     </row>
@@ -14287,7 +14291,7 @@
       <c r="B235" s="50" t="s">
         <v>100</v>
       </c>
-      <c r="C235" s="71" t="s">
+      <c r="C235" s="68" t="s">
         <v>830</v>
       </c>
       <c r="D235" s="52" t="s">
@@ -14309,10 +14313,10 @@
       <c r="J235" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="K235" s="69">
+      <c r="K235" s="66">
         <v>46210.513888888891</v>
       </c>
-      <c r="L235" s="69">
+      <c r="L235" s="66">
         <v>46210.51458333333</v>
       </c>
     </row>
@@ -14323,7 +14327,7 @@
       <c r="B236" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="C236" s="71" t="s">
+      <c r="C236" s="68" t="s">
         <v>832</v>
       </c>
       <c r="D236" s="52" t="s">
@@ -14345,10 +14349,10 @@
       <c r="J236" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="K236" s="69">
+      <c r="K236" s="66">
         <v>46210.061111111114</v>
       </c>
-      <c r="L236" s="69">
+      <c r="L236" s="66">
         <v>46210.460416666669</v>
       </c>
     </row>
@@ -14359,7 +14363,7 @@
       <c r="B237" s="50" t="s">
         <v>266</v>
       </c>
-      <c r="C237" s="71" t="s">
+      <c r="C237" s="68" t="s">
         <v>834</v>
       </c>
       <c r="D237" s="52" t="s">
@@ -14381,10 +14385,10 @@
       <c r="J237" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="K237" s="69">
+      <c r="K237" s="66">
         <v>46208.613888888889</v>
       </c>
-      <c r="L237" s="69">
+      <c r="L237" s="66">
         <v>46209.37777777778</v>
       </c>
     </row>
@@ -14418,21 +14422,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="78" t="s">
         <v>687</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="24" t="s">
@@ -14476,21 +14480,21 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="79" t="s">
         <v>688</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="79"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="79"/>
+      <c r="F4" s="79"/>
+      <c r="G4" s="79"/>
+      <c r="H4" s="79"/>
+      <c r="I4" s="79"/>
+      <c r="J4" s="79"/>
+      <c r="K4" s="79"/>
+      <c r="L4" s="79"/>
+      <c r="M4" s="79"/>
     </row>
     <row r="5" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -14576,7 +14580,7 @@
       </c>
     </row>
     <row r="8" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="81" t="s">
         <v>93</v>
       </c>
       <c r="B8" s="8"/>
@@ -14695,21 +14699,21 @@
       </c>
     </row>
     <row r="11" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="68" t="s">
+      <c r="A11" s="79" t="s">
         <v>689</v>
       </c>
-      <c r="B11" s="68"/>
-      <c r="C11" s="68"/>
-      <c r="D11" s="68"/>
-      <c r="E11" s="68"/>
-      <c r="F11" s="68"/>
-      <c r="G11" s="68"/>
-      <c r="H11" s="68"/>
-      <c r="I11" s="68"/>
-      <c r="J11" s="68"/>
-      <c r="K11" s="68"/>
-      <c r="L11" s="68"/>
-      <c r="M11" s="68"/>
+      <c r="B11" s="79"/>
+      <c r="C11" s="79"/>
+      <c r="D11" s="79"/>
+      <c r="E11" s="79"/>
+      <c r="F11" s="79"/>
+      <c r="G11" s="79"/>
+      <c r="H11" s="79"/>
+      <c r="I11" s="79"/>
+      <c r="J11" s="79"/>
+      <c r="K11" s="79"/>
+      <c r="L11" s="79"/>
+      <c r="M11" s="79"/>
     </row>
     <row r="12" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="25" t="s">
@@ -14905,21 +14909,21 @@
       <c r="M16" s="8"/>
     </row>
     <row r="17" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="68" t="s">
+      <c r="A17" s="79" t="s">
         <v>690</v>
       </c>
-      <c r="B17" s="68"/>
-      <c r="C17" s="68"/>
-      <c r="D17" s="68"/>
-      <c r="E17" s="68"/>
-      <c r="F17" s="68"/>
-      <c r="G17" s="68"/>
-      <c r="H17" s="68"/>
-      <c r="I17" s="68"/>
-      <c r="J17" s="68"/>
-      <c r="K17" s="68"/>
-      <c r="L17" s="68"/>
-      <c r="M17" s="68"/>
+      <c r="B17" s="79"/>
+      <c r="C17" s="79"/>
+      <c r="D17" s="79"/>
+      <c r="E17" s="79"/>
+      <c r="F17" s="79"/>
+      <c r="G17" s="79"/>
+      <c r="H17" s="79"/>
+      <c r="I17" s="79"/>
+      <c r="J17" s="79"/>
+      <c r="K17" s="79"/>
+      <c r="L17" s="79"/>
+      <c r="M17" s="79"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="25" t="s">
@@ -15341,21 +15345,21 @@
       <c r="M28" s="8"/>
     </row>
     <row r="29" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="68" t="s">
+      <c r="A29" s="79" t="s">
         <v>691</v>
       </c>
-      <c r="B29" s="68"/>
-      <c r="C29" s="68"/>
-      <c r="D29" s="68"/>
-      <c r="E29" s="68"/>
-      <c r="F29" s="68"/>
-      <c r="G29" s="68"/>
-      <c r="H29" s="68"/>
-      <c r="I29" s="68"/>
-      <c r="J29" s="68"/>
-      <c r="K29" s="68"/>
-      <c r="L29" s="68"/>
-      <c r="M29" s="68"/>
+      <c r="B29" s="79"/>
+      <c r="C29" s="79"/>
+      <c r="D29" s="79"/>
+      <c r="E29" s="79"/>
+      <c r="F29" s="79"/>
+      <c r="G29" s="79"/>
+      <c r="H29" s="79"/>
+      <c r="I29" s="79"/>
+      <c r="J29" s="79"/>
+      <c r="K29" s="79"/>
+      <c r="L29" s="79"/>
+      <c r="M29" s="79"/>
     </row>
     <row r="30" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A30" s="25" t="s">
@@ -15508,21 +15512,21 @@
       <c r="M33" s="8"/>
     </row>
     <row r="34" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="68" t="s">
+      <c r="A34" s="79" t="s">
         <v>692</v>
       </c>
-      <c r="B34" s="68"/>
-      <c r="C34" s="68"/>
-      <c r="D34" s="68"/>
-      <c r="E34" s="68"/>
-      <c r="F34" s="68"/>
-      <c r="G34" s="68"/>
-      <c r="H34" s="68"/>
-      <c r="I34" s="68"/>
-      <c r="J34" s="68"/>
-      <c r="K34" s="68"/>
-      <c r="L34" s="68"/>
-      <c r="M34" s="68"/>
+      <c r="B34" s="79"/>
+      <c r="C34" s="79"/>
+      <c r="D34" s="79"/>
+      <c r="E34" s="79"/>
+      <c r="F34" s="79"/>
+      <c r="G34" s="79"/>
+      <c r="H34" s="79"/>
+      <c r="I34" s="79"/>
+      <c r="J34" s="79"/>
+      <c r="K34" s="79"/>
+      <c r="L34" s="79"/>
+      <c r="M34" s="79"/>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" s="25" t="s">
@@ -15648,21 +15652,21 @@
       </c>
     </row>
     <row r="38" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="68" t="s">
+      <c r="A38" s="79" t="s">
         <v>693</v>
       </c>
-      <c r="B38" s="68"/>
-      <c r="C38" s="68"/>
-      <c r="D38" s="68"/>
-      <c r="E38" s="68"/>
-      <c r="F38" s="68"/>
-      <c r="G38" s="68"/>
-      <c r="H38" s="68"/>
-      <c r="I38" s="68"/>
-      <c r="J38" s="68"/>
-      <c r="K38" s="68"/>
-      <c r="L38" s="68"/>
-      <c r="M38" s="68"/>
+      <c r="B38" s="79"/>
+      <c r="C38" s="79"/>
+      <c r="D38" s="79"/>
+      <c r="E38" s="79"/>
+      <c r="F38" s="79"/>
+      <c r="G38" s="79"/>
+      <c r="H38" s="79"/>
+      <c r="I38" s="79"/>
+      <c r="J38" s="79"/>
+      <c r="K38" s="79"/>
+      <c r="L38" s="79"/>
+      <c r="M38" s="79"/>
     </row>
     <row r="39" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A39" s="25" t="s">
@@ -16085,21 +16089,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="78" t="s">
         <v>694</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -16143,21 +16147,21 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="79" t="s">
         <v>695</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="79"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="79"/>
+      <c r="F4" s="79"/>
+      <c r="G4" s="79"/>
+      <c r="H4" s="79"/>
+      <c r="I4" s="79"/>
+      <c r="J4" s="79"/>
+      <c r="K4" s="79"/>
+      <c r="L4" s="79"/>
+      <c r="M4" s="79"/>
     </row>
     <row r="5" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
@@ -16478,21 +16482,21 @@
       <c r="M12" s="8"/>
     </row>
     <row r="13" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="68" t="s">
+      <c r="A13" s="79" t="s">
         <v>696</v>
       </c>
-      <c r="B13" s="68"/>
-      <c r="C13" s="68"/>
-      <c r="D13" s="68"/>
-      <c r="E13" s="68"/>
-      <c r="F13" s="68"/>
-      <c r="G13" s="68"/>
-      <c r="H13" s="68"/>
-      <c r="I13" s="68"/>
-      <c r="J13" s="68"/>
-      <c r="K13" s="68"/>
-      <c r="L13" s="68"/>
-      <c r="M13" s="68"/>
+      <c r="B13" s="79"/>
+      <c r="C13" s="79"/>
+      <c r="D13" s="79"/>
+      <c r="E13" s="79"/>
+      <c r="F13" s="79"/>
+      <c r="G13" s="79"/>
+      <c r="H13" s="79"/>
+      <c r="I13" s="79"/>
+      <c r="J13" s="79"/>
+      <c r="K13" s="79"/>
+      <c r="L13" s="79"/>
+      <c r="M13" s="79"/>
     </row>
     <row r="14" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
@@ -16536,21 +16540,21 @@
       </c>
     </row>
     <row r="15" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="68" t="s">
+      <c r="A15" s="79" t="s">
         <v>697</v>
       </c>
-      <c r="B15" s="68"/>
-      <c r="C15" s="68"/>
-      <c r="D15" s="68"/>
-      <c r="E15" s="68"/>
-      <c r="F15" s="68"/>
-      <c r="G15" s="68"/>
-      <c r="H15" s="68"/>
-      <c r="I15" s="68"/>
-      <c r="J15" s="68"/>
-      <c r="K15" s="68"/>
-      <c r="L15" s="68"/>
-      <c r="M15" s="68"/>
+      <c r="B15" s="79"/>
+      <c r="C15" s="79"/>
+      <c r="D15" s="79"/>
+      <c r="E15" s="79"/>
+      <c r="F15" s="79"/>
+      <c r="G15" s="79"/>
+      <c r="H15" s="79"/>
+      <c r="I15" s="79"/>
+      <c r="J15" s="79"/>
+      <c r="K15" s="79"/>
+      <c r="L15" s="79"/>
+      <c r="M15" s="79"/>
     </row>
     <row r="16" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
@@ -16676,21 +16680,21 @@
       </c>
     </row>
     <row r="19" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="68" t="s">
+      <c r="A19" s="79" t="s">
         <v>698</v>
       </c>
-      <c r="B19" s="68"/>
-      <c r="C19" s="68"/>
-      <c r="D19" s="68"/>
-      <c r="E19" s="68"/>
-      <c r="F19" s="68"/>
-      <c r="G19" s="68"/>
-      <c r="H19" s="68"/>
-      <c r="I19" s="68"/>
-      <c r="J19" s="68"/>
-      <c r="K19" s="68"/>
-      <c r="L19" s="68"/>
-      <c r="M19" s="68"/>
+      <c r="B19" s="79"/>
+      <c r="C19" s="79"/>
+      <c r="D19" s="79"/>
+      <c r="E19" s="79"/>
+      <c r="F19" s="79"/>
+      <c r="G19" s="79"/>
+      <c r="H19" s="79"/>
+      <c r="I19" s="79"/>
+      <c r="J19" s="79"/>
+      <c r="K19" s="79"/>
+      <c r="L19" s="79"/>
+      <c r="M19" s="79"/>
     </row>
     <row r="20" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
@@ -16730,21 +16734,21 @@
       <c r="M20" s="8"/>
     </row>
     <row r="21" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="68" t="s">
+      <c r="A21" s="79" t="s">
         <v>699</v>
       </c>
-      <c r="B21" s="68"/>
-      <c r="C21" s="68"/>
-      <c r="D21" s="68"/>
-      <c r="E21" s="68"/>
-      <c r="F21" s="68"/>
-      <c r="G21" s="68"/>
-      <c r="H21" s="68"/>
-      <c r="I21" s="68"/>
-      <c r="J21" s="68"/>
-      <c r="K21" s="68"/>
-      <c r="L21" s="68"/>
-      <c r="M21" s="68"/>
+      <c r="B21" s="79"/>
+      <c r="C21" s="79"/>
+      <c r="D21" s="79"/>
+      <c r="E21" s="79"/>
+      <c r="F21" s="79"/>
+      <c r="G21" s="79"/>
+      <c r="H21" s="79"/>
+      <c r="I21" s="79"/>
+      <c r="J21" s="79"/>
+      <c r="K21" s="79"/>
+      <c r="L21" s="79"/>
+      <c r="M21" s="79"/>
     </row>
     <row r="22" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
@@ -16980,21 +16984,21 @@
       </c>
     </row>
     <row r="28" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="68" t="s">
+      <c r="A28" s="79" t="s">
         <v>700</v>
       </c>
-      <c r="B28" s="68"/>
-      <c r="C28" s="68"/>
-      <c r="D28" s="68"/>
-      <c r="E28" s="68"/>
-      <c r="F28" s="68"/>
-      <c r="G28" s="68"/>
-      <c r="H28" s="68"/>
-      <c r="I28" s="68"/>
-      <c r="J28" s="68"/>
-      <c r="K28" s="68"/>
-      <c r="L28" s="68"/>
-      <c r="M28" s="68"/>
+      <c r="B28" s="79"/>
+      <c r="C28" s="79"/>
+      <c r="D28" s="79"/>
+      <c r="E28" s="79"/>
+      <c r="F28" s="79"/>
+      <c r="G28" s="79"/>
+      <c r="H28" s="79"/>
+      <c r="I28" s="79"/>
+      <c r="J28" s="79"/>
+      <c r="K28" s="79"/>
+      <c r="L28" s="79"/>
+      <c r="M28" s="79"/>
     </row>
     <row r="29" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
@@ -18431,7 +18435,7 @@
       <c r="B65" s="50" t="s">
         <v>100</v>
       </c>
-      <c r="C65" s="71" t="s">
+      <c r="C65" s="68" t="s">
         <v>824</v>
       </c>
       <c r="D65" s="52" t="s">
@@ -18453,10 +18457,10 @@
       <c r="J65" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="K65" s="69">
+      <c r="K65" s="66">
         <v>46211.036805555559</v>
       </c>
-      <c r="L65" s="69">
+      <c r="L65" s="66">
         <v>46211.036805555559</v>
       </c>
     </row>
@@ -18500,21 +18504,21 @@
       </c>
     </row>
     <row r="67" spans="1:13" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="68" t="s">
+      <c r="A67" s="79" t="s">
         <v>701</v>
       </c>
-      <c r="B67" s="68"/>
-      <c r="C67" s="68"/>
-      <c r="D67" s="68"/>
-      <c r="E67" s="68"/>
-      <c r="F67" s="68"/>
-      <c r="G67" s="68"/>
-      <c r="H67" s="68"/>
-      <c r="I67" s="68"/>
-      <c r="J67" s="68"/>
-      <c r="K67" s="68"/>
-      <c r="L67" s="68"/>
-      <c r="M67" s="68"/>
+      <c r="B67" s="79"/>
+      <c r="C67" s="79"/>
+      <c r="D67" s="79"/>
+      <c r="E67" s="79"/>
+      <c r="F67" s="79"/>
+      <c r="G67" s="79"/>
+      <c r="H67" s="79"/>
+      <c r="I67" s="79"/>
+      <c r="J67" s="79"/>
+      <c r="K67" s="79"/>
+      <c r="L67" s="79"/>
+      <c r="M67" s="79"/>
     </row>
     <row r="68" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A68" s="8" t="s">
@@ -18636,7 +18640,7 @@
       <c r="A74" s="23" t="s">
         <v>759</v>
       </c>
-      <c r="C74" s="72" t="s">
+      <c r="C74" s="69" t="s">
         <v>756</v>
       </c>
       <c r="D74" s="59" t="s">
@@ -18647,7 +18651,7 @@
       <c r="A75" s="23" t="s">
         <v>759</v>
       </c>
-      <c r="C75" s="72" t="s">
+      <c r="C75" s="69" t="s">
         <v>777</v>
       </c>
       <c r="D75" s="59" t="s">
@@ -18655,7 +18659,7 @@
       </c>
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="C76" s="72" t="s">
+      <c r="C76" s="69" t="s">
         <v>757</v>
       </c>
       <c r="D76" s="59" t="s">
@@ -18663,7 +18667,7 @@
       </c>
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="C77" s="72" t="s">
+      <c r="C77" s="69" t="s">
         <v>772</v>
       </c>
       <c r="D77" s="59" t="s">
@@ -18671,7 +18675,7 @@
       </c>
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="C78" s="72" t="s">
+      <c r="C78" s="69" t="s">
         <v>762</v>
       </c>
       <c r="D78" s="59" t="s">
@@ -18679,7 +18683,7 @@
       </c>
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="C79" s="72" t="s">
+      <c r="C79" s="69" t="s">
         <v>763</v>
       </c>
       <c r="D79" s="59" t="s">
@@ -18687,7 +18691,7 @@
       </c>
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="C80" s="72" t="s">
+      <c r="C80" s="69" t="s">
         <v>822</v>
       </c>
       <c r="D80" s="59" t="s">
@@ -18695,13 +18699,13 @@
       </c>
     </row>
     <row r="81" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C81" s="73" t="s">
+      <c r="C81" s="70" t="s">
         <v>836</v>
       </c>
       <c r="D81" s="59"/>
     </row>
     <row r="82" spans="3:4" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="C82" s="72" t="s">
+      <c r="C82" s="69" t="s">
         <v>792</v>
       </c>
       <c r="D82" s="59" t="s">
@@ -18709,13 +18713,13 @@
       </c>
     </row>
     <row r="83" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C83" s="73" t="s">
+      <c r="C83" s="70" t="s">
         <v>821</v>
       </c>
       <c r="D83" s="59"/>
     </row>
     <row r="84" spans="3:4" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="C84" s="74" t="s">
+      <c r="C84" s="71" t="s">
         <v>791</v>
       </c>
       <c r="D84" s="63" t="s">
@@ -18723,7 +18727,7 @@
       </c>
     </row>
     <row r="85" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C85" s="72" t="s">
+      <c r="C85" s="69" t="s">
         <v>819</v>
       </c>
       <c r="D85" s="59" t="s">
@@ -18731,7 +18735,7 @@
       </c>
     </row>
     <row r="86" spans="3:4" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="C86" s="72" t="s">
+      <c r="C86" s="69" t="s">
         <v>767</v>
       </c>
       <c r="D86" s="59" t="s">
@@ -18787,21 +18791,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="78" t="s">
         <v>702</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -18845,21 +18849,21 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="79" t="s">
         <v>703</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="79"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="79"/>
+      <c r="F4" s="79"/>
+      <c r="G4" s="79"/>
+      <c r="H4" s="79"/>
+      <c r="I4" s="79"/>
+      <c r="J4" s="79"/>
+      <c r="K4" s="79"/>
+      <c r="L4" s="79"/>
+      <c r="M4" s="79"/>
     </row>
     <row r="5" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
@@ -18903,21 +18907,21 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="68" t="s">
+      <c r="A6" s="79" t="s">
         <v>704</v>
       </c>
-      <c r="B6" s="68"/>
-      <c r="C6" s="68"/>
-      <c r="D6" s="68"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="68"/>
-      <c r="H6" s="68"/>
-      <c r="I6" s="68"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="68"/>
-      <c r="L6" s="68"/>
-      <c r="M6" s="68"/>
+      <c r="B6" s="79"/>
+      <c r="C6" s="79"/>
+      <c r="D6" s="79"/>
+      <c r="E6" s="79"/>
+      <c r="F6" s="79"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
+      <c r="I6" s="79"/>
+      <c r="J6" s="79"/>
+      <c r="K6" s="79"/>
+      <c r="L6" s="79"/>
+      <c r="M6" s="79"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
@@ -19000,21 +19004,21 @@
       </c>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="68" t="s">
+      <c r="A9" s="79" t="s">
         <v>705</v>
       </c>
-      <c r="B9" s="68"/>
-      <c r="C9" s="68"/>
-      <c r="D9" s="68"/>
-      <c r="E9" s="68"/>
-      <c r="F9" s="68"/>
-      <c r="G9" s="68"/>
-      <c r="H9" s="68"/>
-      <c r="I9" s="68"/>
-      <c r="J9" s="68"/>
-      <c r="K9" s="68"/>
-      <c r="L9" s="68"/>
-      <c r="M9" s="68"/>
+      <c r="B9" s="79"/>
+      <c r="C9" s="79"/>
+      <c r="D9" s="79"/>
+      <c r="E9" s="79"/>
+      <c r="F9" s="79"/>
+      <c r="G9" s="79"/>
+      <c r="H9" s="79"/>
+      <c r="I9" s="79"/>
+      <c r="J9" s="79"/>
+      <c r="K9" s="79"/>
+      <c r="L9" s="79"/>
+      <c r="M9" s="79"/>
     </row>
     <row r="10" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
@@ -19171,21 +19175,21 @@
       <c r="M13" s="8"/>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="68" t="s">
+      <c r="A14" s="79" t="s">
         <v>706</v>
       </c>
-      <c r="B14" s="68"/>
-      <c r="C14" s="68"/>
-      <c r="D14" s="68"/>
-      <c r="E14" s="68"/>
-      <c r="F14" s="68"/>
-      <c r="G14" s="68"/>
-      <c r="H14" s="68"/>
-      <c r="I14" s="68"/>
-      <c r="J14" s="68"/>
-      <c r="K14" s="68"/>
-      <c r="L14" s="68"/>
-      <c r="M14" s="68"/>
+      <c r="B14" s="79"/>
+      <c r="C14" s="79"/>
+      <c r="D14" s="79"/>
+      <c r="E14" s="79"/>
+      <c r="F14" s="79"/>
+      <c r="G14" s="79"/>
+      <c r="H14" s="79"/>
+      <c r="I14" s="79"/>
+      <c r="J14" s="79"/>
+      <c r="K14" s="79"/>
+      <c r="L14" s="79"/>
+      <c r="M14" s="79"/>
     </row>
     <row r="15" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
@@ -19225,21 +19229,21 @@
       <c r="M15" s="8"/>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="68" t="s">
+      <c r="A16" s="79" t="s">
         <v>707</v>
       </c>
-      <c r="B16" s="68"/>
-      <c r="C16" s="68"/>
-      <c r="D16" s="68"/>
-      <c r="E16" s="68"/>
-      <c r="F16" s="68"/>
-      <c r="G16" s="68"/>
-      <c r="H16" s="68"/>
-      <c r="I16" s="68"/>
-      <c r="J16" s="68"/>
-      <c r="K16" s="68"/>
-      <c r="L16" s="68"/>
-      <c r="M16" s="68"/>
+      <c r="B16" s="79"/>
+      <c r="C16" s="79"/>
+      <c r="D16" s="79"/>
+      <c r="E16" s="79"/>
+      <c r="F16" s="79"/>
+      <c r="G16" s="79"/>
+      <c r="H16" s="79"/>
+      <c r="I16" s="79"/>
+      <c r="J16" s="79"/>
+      <c r="K16" s="79"/>
+      <c r="L16" s="79"/>
+      <c r="M16" s="79"/>
     </row>
     <row r="17" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
@@ -19439,21 +19443,21 @@
       </c>
     </row>
     <row r="22" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="68" t="s">
+      <c r="A22" s="79" t="s">
         <v>708</v>
       </c>
-      <c r="B22" s="68"/>
-      <c r="C22" s="68"/>
-      <c r="D22" s="68"/>
-      <c r="E22" s="68"/>
-      <c r="F22" s="68"/>
-      <c r="G22" s="68"/>
-      <c r="H22" s="68"/>
-      <c r="I22" s="68"/>
-      <c r="J22" s="68"/>
-      <c r="K22" s="68"/>
-      <c r="L22" s="68"/>
-      <c r="M22" s="68"/>
+      <c r="B22" s="79"/>
+      <c r="C22" s="79"/>
+      <c r="D22" s="79"/>
+      <c r="E22" s="79"/>
+      <c r="F22" s="79"/>
+      <c r="G22" s="79"/>
+      <c r="H22" s="79"/>
+      <c r="I22" s="79"/>
+      <c r="J22" s="79"/>
+      <c r="K22" s="79"/>
+      <c r="L22" s="79"/>
+      <c r="M22" s="79"/>
     </row>
     <row r="23" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
@@ -19678,13 +19682,13 @@
       <c r="M28" s="8"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A29" s="50" t="s">
+      <c r="A29" s="80" t="s">
         <v>831</v>
       </c>
       <c r="B29" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="C29" s="71" t="s">
+      <c r="C29" s="68" t="s">
         <v>832</v>
       </c>
       <c r="D29" s="52" t="s">
@@ -19706,10 +19710,10 @@
       <c r="J29" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="K29" s="69">
+      <c r="K29" s="66">
         <v>46210.061111111114</v>
       </c>
-      <c r="L29" s="69">
+      <c r="L29" s="66">
         <v>46210.460416666669</v>
       </c>
     </row>
@@ -19751,21 +19755,21 @@
       <c r="M30" s="8"/>
     </row>
     <row r="31" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="68" t="s">
+      <c r="A31" s="79" t="s">
         <v>709</v>
       </c>
-      <c r="B31" s="68"/>
-      <c r="C31" s="68"/>
-      <c r="D31" s="68"/>
-      <c r="E31" s="68"/>
-      <c r="F31" s="68"/>
-      <c r="G31" s="68"/>
-      <c r="H31" s="68"/>
-      <c r="I31" s="68"/>
-      <c r="J31" s="68"/>
-      <c r="K31" s="68"/>
-      <c r="L31" s="68"/>
-      <c r="M31" s="68"/>
+      <c r="B31" s="79"/>
+      <c r="C31" s="79"/>
+      <c r="D31" s="79"/>
+      <c r="E31" s="79"/>
+      <c r="F31" s="79"/>
+      <c r="G31" s="79"/>
+      <c r="H31" s="79"/>
+      <c r="I31" s="79"/>
+      <c r="J31" s="79"/>
+      <c r="K31" s="79"/>
+      <c r="L31" s="79"/>
+      <c r="M31" s="79"/>
     </row>
     <row r="32" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
@@ -19881,21 +19885,21 @@
       <c r="M34" s="8"/>
     </row>
     <row r="35" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="68" t="s">
+      <c r="A35" s="79" t="s">
         <v>710</v>
       </c>
-      <c r="B35" s="68"/>
-      <c r="C35" s="68"/>
-      <c r="D35" s="68"/>
-      <c r="E35" s="68"/>
-      <c r="F35" s="68"/>
-      <c r="G35" s="68"/>
-      <c r="H35" s="68"/>
-      <c r="I35" s="68"/>
-      <c r="J35" s="68"/>
-      <c r="K35" s="68"/>
-      <c r="L35" s="68"/>
-      <c r="M35" s="68"/>
+      <c r="B35" s="79"/>
+      <c r="C35" s="79"/>
+      <c r="D35" s="79"/>
+      <c r="E35" s="79"/>
+      <c r="F35" s="79"/>
+      <c r="G35" s="79"/>
+      <c r="H35" s="79"/>
+      <c r="I35" s="79"/>
+      <c r="J35" s="79"/>
+      <c r="K35" s="79"/>
+      <c r="L35" s="79"/>
+      <c r="M35" s="79"/>
     </row>
     <row r="36" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
@@ -20505,7 +20509,7 @@
       <c r="B52" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="C52" s="71" t="s">
+      <c r="C52" s="68" t="s">
         <v>828</v>
       </c>
       <c r="D52" s="52" t="s">
@@ -20527,10 +20531,10 @@
       <c r="J52" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="K52" s="69">
+      <c r="K52" s="66">
         <v>46210.981944444444</v>
       </c>
-      <c r="L52" s="69">
+      <c r="L52" s="66">
         <v>46210.981944444444</v>
       </c>
     </row>
@@ -20572,21 +20576,21 @@
       <c r="M53" s="8"/>
     </row>
     <row r="54" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="68" t="s">
+      <c r="A54" s="79" t="s">
         <v>711</v>
       </c>
-      <c r="B54" s="68"/>
-      <c r="C54" s="68"/>
-      <c r="D54" s="68"/>
-      <c r="E54" s="68"/>
-      <c r="F54" s="68"/>
-      <c r="G54" s="68"/>
-      <c r="H54" s="68"/>
-      <c r="I54" s="68"/>
-      <c r="J54" s="68"/>
-      <c r="K54" s="68"/>
-      <c r="L54" s="68"/>
-      <c r="M54" s="68"/>
+      <c r="B54" s="79"/>
+      <c r="C54" s="79"/>
+      <c r="D54" s="79"/>
+      <c r="E54" s="79"/>
+      <c r="F54" s="79"/>
+      <c r="G54" s="79"/>
+      <c r="H54" s="79"/>
+      <c r="I54" s="79"/>
+      <c r="J54" s="79"/>
+      <c r="K54" s="79"/>
+      <c r="L54" s="79"/>
+      <c r="M54" s="79"/>
     </row>
     <row r="55" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A55" s="8" t="s">
@@ -20626,21 +20630,21 @@
       <c r="M55" s="8"/>
     </row>
     <row r="56" spans="1:13" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="68" t="s">
+      <c r="A56" s="79" t="s">
         <v>712</v>
       </c>
-      <c r="B56" s="68"/>
-      <c r="C56" s="68"/>
-      <c r="D56" s="68"/>
-      <c r="E56" s="68"/>
-      <c r="F56" s="68"/>
-      <c r="G56" s="68"/>
-      <c r="H56" s="68"/>
-      <c r="I56" s="68"/>
-      <c r="J56" s="68"/>
-      <c r="K56" s="68"/>
-      <c r="L56" s="68"/>
-      <c r="M56" s="68"/>
+      <c r="B56" s="79"/>
+      <c r="C56" s="79"/>
+      <c r="D56" s="79"/>
+      <c r="E56" s="79"/>
+      <c r="F56" s="79"/>
+      <c r="G56" s="79"/>
+      <c r="H56" s="79"/>
+      <c r="I56" s="79"/>
+      <c r="J56" s="79"/>
+      <c r="K56" s="79"/>
+      <c r="L56" s="79"/>
+      <c r="M56" s="79"/>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" s="8" t="s">
@@ -20713,7 +20717,7 @@
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="C62" s="75" t="s">
+      <c r="C62" s="72" t="s">
         <v>838</v>
       </c>
       <c r="D62" s="46"/>
@@ -20722,7 +20726,7 @@
       <c r="C63" s="60" t="s">
         <v>779</v>
       </c>
-      <c r="D63" s="79" t="s">
+      <c r="D63" s="76" t="s">
         <v>774</v>
       </c>
     </row>
@@ -20730,18 +20734,18 @@
       <c r="C64" s="46" t="s">
         <v>780</v>
       </c>
-      <c r="D64" s="76" t="s">
+      <c r="D64" s="73" t="s">
         <v>776</v>
       </c>
     </row>
     <row r="65" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C65" s="77" t="s">
+      <c r="C65" s="74" t="s">
         <v>783</v>
       </c>
       <c r="D65" s="46"/>
     </row>
     <row r="66" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C66" s="78" t="s">
+      <c r="C66" s="75" t="s">
         <v>784</v>
       </c>
       <c r="D66" s="46" t="s">
@@ -20749,7 +20753,7 @@
       </c>
     </row>
     <row r="67" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C67" s="78" t="s">
+      <c r="C67" s="75" t="s">
         <v>839</v>
       </c>
       <c r="D67" s="46" t="s">
@@ -20766,17 +20770,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="A9:M9"/>
+    <mergeCell ref="A14:M14"/>
     <mergeCell ref="A56:M56"/>
     <mergeCell ref="A16:M16"/>
     <mergeCell ref="A22:M22"/>
     <mergeCell ref="A31:M31"/>
     <mergeCell ref="A35:M35"/>
     <mergeCell ref="A54:M54"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="A6:M6"/>
-    <mergeCell ref="A9:M9"/>
-    <mergeCell ref="A14:M14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D64" r:id="rId1" xr:uid="{5086776A-0A7E-4AED-AE41-2F854BC2FEE7}"/>
@@ -20805,21 +20809,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="78" t="s">
         <v>713</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -20863,21 +20867,21 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="79" t="s">
         <v>714</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="79"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="79"/>
+      <c r="F4" s="79"/>
+      <c r="G4" s="79"/>
+      <c r="H4" s="79"/>
+      <c r="I4" s="79"/>
+      <c r="J4" s="79"/>
+      <c r="K4" s="79"/>
+      <c r="L4" s="79"/>
+      <c r="M4" s="79"/>
     </row>
     <row r="5" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
@@ -21293,21 +21297,21 @@
       <c r="M15" s="8"/>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="68" t="s">
+      <c r="A16" s="79" t="s">
         <v>715</v>
       </c>
-      <c r="B16" s="68"/>
-      <c r="C16" s="68"/>
-      <c r="D16" s="68"/>
-      <c r="E16" s="68"/>
-      <c r="F16" s="68"/>
-      <c r="G16" s="68"/>
-      <c r="H16" s="68"/>
-      <c r="I16" s="68"/>
-      <c r="J16" s="68"/>
-      <c r="K16" s="68"/>
-      <c r="L16" s="68"/>
-      <c r="M16" s="68"/>
+      <c r="B16" s="79"/>
+      <c r="C16" s="79"/>
+      <c r="D16" s="79"/>
+      <c r="E16" s="79"/>
+      <c r="F16" s="79"/>
+      <c r="G16" s="79"/>
+      <c r="H16" s="79"/>
+      <c r="I16" s="79"/>
+      <c r="J16" s="79"/>
+      <c r="K16" s="79"/>
+      <c r="L16" s="79"/>
+      <c r="M16" s="79"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
@@ -21990,7 +21994,7 @@
       <c r="B35" s="50" t="s">
         <v>100</v>
       </c>
-      <c r="C35" s="71" t="s">
+      <c r="C35" s="68" t="s">
         <v>826</v>
       </c>
       <c r="D35" s="52" t="s">
@@ -22012,10 +22016,10 @@
       <c r="J35" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="K35" s="69">
+      <c r="K35" s="66">
         <v>46210.98541666667</v>
       </c>
-      <c r="L35" s="69">
+      <c r="L35" s="66">
         <v>46210.98541666667</v>
       </c>
     </row>
@@ -22057,21 +22061,21 @@
       <c r="M36" s="8"/>
     </row>
     <row r="37" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="68" t="s">
+      <c r="A37" s="79" t="s">
         <v>716</v>
       </c>
-      <c r="B37" s="68"/>
-      <c r="C37" s="68"/>
-      <c r="D37" s="68"/>
-      <c r="E37" s="68"/>
-      <c r="F37" s="68"/>
-      <c r="G37" s="68"/>
-      <c r="H37" s="68"/>
-      <c r="I37" s="68"/>
-      <c r="J37" s="68"/>
-      <c r="K37" s="68"/>
-      <c r="L37" s="68"/>
-      <c r="M37" s="68"/>
+      <c r="B37" s="79"/>
+      <c r="C37" s="79"/>
+      <c r="D37" s="79"/>
+      <c r="E37" s="79"/>
+      <c r="F37" s="79"/>
+      <c r="G37" s="79"/>
+      <c r="H37" s="79"/>
+      <c r="I37" s="79"/>
+      <c r="J37" s="79"/>
+      <c r="K37" s="79"/>
+      <c r="L37" s="79"/>
+      <c r="M37" s="79"/>
     </row>
     <row r="38" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A38" s="8" t="s">
@@ -22709,21 +22713,21 @@
       <c r="M54" s="8"/>
     </row>
     <row r="55" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="68" t="s">
+      <c r="A55" s="79" t="s">
         <v>717</v>
       </c>
-      <c r="B55" s="68"/>
-      <c r="C55" s="68"/>
-      <c r="D55" s="68"/>
-      <c r="E55" s="68"/>
-      <c r="F55" s="68"/>
-      <c r="G55" s="68"/>
-      <c r="H55" s="68"/>
-      <c r="I55" s="68"/>
-      <c r="J55" s="68"/>
-      <c r="K55" s="68"/>
-      <c r="L55" s="68"/>
-      <c r="M55" s="68"/>
+      <c r="B55" s="79"/>
+      <c r="C55" s="79"/>
+      <c r="D55" s="79"/>
+      <c r="E55" s="79"/>
+      <c r="F55" s="79"/>
+      <c r="G55" s="79"/>
+      <c r="H55" s="79"/>
+      <c r="I55" s="79"/>
+      <c r="J55" s="79"/>
+      <c r="K55" s="79"/>
+      <c r="L55" s="79"/>
+      <c r="M55" s="79"/>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" s="8" t="s">
@@ -23635,7 +23639,7 @@
       <c r="B79" s="50" t="s">
         <v>100</v>
       </c>
-      <c r="C79" s="71" t="s">
+      <c r="C79" s="68" t="s">
         <v>830</v>
       </c>
       <c r="D79" s="52" t="s">
@@ -23657,10 +23661,10 @@
       <c r="J79" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="K79" s="69">
+      <c r="K79" s="66">
         <v>46210.513888888891</v>
       </c>
-      <c r="L79" s="69">
+      <c r="L79" s="66">
         <v>46210.51458333333</v>
       </c>
     </row>
@@ -23671,7 +23675,7 @@
       <c r="B80" s="50" t="s">
         <v>266</v>
       </c>
-      <c r="C80" s="71" t="s">
+      <c r="C80" s="68" t="s">
         <v>834</v>
       </c>
       <c r="D80" s="52" t="s">
@@ -23693,10 +23697,10 @@
       <c r="J80" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="K80" s="69">
+      <c r="K80" s="66">
         <v>46208.613888888889</v>
       </c>
-      <c r="L80" s="69">
+      <c r="L80" s="66">
         <v>46209.37777777778</v>
       </c>
     </row>
@@ -23807,21 +23811,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="78" t="s">
         <v>718</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -23865,21 +23869,21 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="79" t="s">
         <v>719</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="79"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="79"/>
+      <c r="F4" s="79"/>
+      <c r="G4" s="79"/>
+      <c r="H4" s="79"/>
+      <c r="I4" s="79"/>
+      <c r="J4" s="79"/>
+      <c r="K4" s="79"/>
+      <c r="L4" s="79"/>
+      <c r="M4" s="79"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">

</xml_diff>